<commit_message>
Add realistic invoice payment statuses
</commit_message>
<xml_diff>
--- a/invoices/invoice_2026-01-01.xlsx
+++ b/invoices/invoice_2026-01-01.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F27"/>
+  <dimension ref="B2:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -610,7 +610,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>PAID</t>
         </is>
       </c>
     </row>
@@ -694,14 +694,14 @@
     <row r="16" ht="28" customHeight="1">
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Data Analysis &amp; Reporting</t>
+          <t>UI/UX Design Services</t>
         </is>
       </c>
       <c r="C16" s="12" t="n">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>600000</v>
+        <v>750000</v>
       </c>
       <c r="E16" s="14" t="n">
         <v>0.11</v>
@@ -714,14 +714,14 @@
     <row r="17" ht="28" customHeight="1">
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>UI/UX Design Services</t>
+          <t>Project Management</t>
         </is>
       </c>
       <c r="C17" s="12" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D17" s="13" t="n">
-        <v>750000</v>
+        <v>450000</v>
       </c>
       <c r="E17" s="14" t="n">
         <v>0.11</v>
@@ -731,48 +731,68 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="D19" s="15" t="inlineStr">
-        <is>
-          <t>Subtotal:</t>
-        </is>
-      </c>
-      <c r="F19" s="13">
-        <f>SUMPRODUCT(C16:C17,D16:D17)</f>
+    <row r="18" ht="28" customHeight="1">
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>System Integration &amp; Testing</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="n">
+        <v>44</v>
+      </c>
+      <c r="D18" s="13" t="n">
+        <v>400000</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F18" s="13">
+        <f>C18*D18*(1+E18)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="D20" s="15" t="inlineStr">
         <is>
+          <t>Subtotal:</t>
+        </is>
+      </c>
+      <c r="F20" s="13">
+        <f>SUMPRODUCT(C16:C18,D16:D18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="D21" s="15" t="inlineStr">
+        <is>
           <t>Tax (11%):</t>
         </is>
       </c>
-      <c r="F20" s="13">
-        <f>SUMPRODUCT(C16:C17,D16:D17,E16:E17)</f>
+      <c r="F21" s="13">
+        <f>SUMPRODUCT(C16:C18,D16:D18,E16:E18)</f>
         <v/>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="D21" s="16" t="inlineStr">
+    <row r="22" ht="24" customHeight="1">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>TOTAL DUE:</t>
         </is>
       </c>
-      <c r="F21" s="17">
-        <f>F19+F20</f>
+      <c r="F22" s="17">
+        <f>F20+F21</f>
         <v/>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="7" t="inlineStr">
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>PAYMENT TERMS &amp; NOTES</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="50" customHeight="1">
-      <c r="B25" s="11" t="inlineStr">
+    <row r="26" ht="50" customHeight="1">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>• Payment terms: Net 30 days from invoice date
 • Please transfer to Bank Mandiri, Account: 123-456-789
@@ -780,8 +800,8 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="B27" s="18" t="inlineStr">
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>This is an electronically generated invoice. No signature required.</t>
         </is>
@@ -790,14 +810,14 @@
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="C13:F13"/>
-    <mergeCell ref="B24:F24"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B25:F25"/>
     <mergeCell ref="C12:F12"/>
     <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B28:F28"/>
     <mergeCell ref="C11:F11"/>
-    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B26:F26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>